<commit_message>
Fill About, contact, How I work and Build log; add link previews; fix audit issues
- Set email, About text and the four How I work steps
- Replace the placeholder log entry with two real entries
- Confirm Claude and Perplexity wording; task AI notes now say Claude created the simulations
- Add Open Graph tags, canonical links and a generated preview image (public/og.png);
  the build fails until `site` is set in astro.config.mjs
- Let image alt text name the full-size image links (screen readers lost it)
- Show the vendor review's result in its title; stop task pages repeating the brief
- Set Excel to daily, use en-GB and UK spelling, fix log.astro attribute spacing
- Replace the starter README
- Update the QA checklist and vendor review sample files

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/samples/vendor-spend-review/vendor-spend-review.xlsx
+++ b/public/samples/vendor-spend-review/vendor-spend-review.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://oagkenya-my.sharepoint.com/personal/eddah_dena_oagkenya_go_ke/Documents/Portolio Workings/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="120" documentId="8_{E8346B1F-E607-47C2-B6B4-94B25FBADFEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B91F5127-591E-4317-94A2-7D351AE32240}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="734" activeTab="1" xr2:uid="{999650B2-D879-4600-8074-8BBEC06EDFB8}"/>

</xml_diff>